<commit_message>
Auto update ETF comparison: Mon Apr 27 10:41:27 UTC 2026
</commit_message>
<xml_diff>
--- a/data/00982A/20260427.xlsx
+++ b/data/00982A/20260427.xlsx
@@ -385,7 +385,7 @@
         <v>基金淨資產價值(元)</v>
       </c>
       <c r="B1" t="str">
-        <v>TWD 38,855,229,625</v>
+        <v>TWD 38,640,824,146</v>
       </c>
     </row>
     <row r="2">
@@ -393,7 +393,7 @@
         <v>每受益權單位淨資產價值(元)-台幣交易</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD 20.86</v>
+        <v>TWD 20.69</v>
       </c>
     </row>
     <row r="3">
@@ -401,7 +401,7 @@
         <v>已發行受益權單位總數-台幣交易</v>
       </c>
       <c r="B3" t="str">
-        <v>1,862,436,000</v>
+        <v>1,867,436,000</v>
       </c>
     </row>
   </sheetData>
@@ -437,7 +437,7 @@
         <v>台積電</v>
       </c>
       <c r="C2" t="str">
-        <v>8.71%</v>
+        <v>9.07%</v>
       </c>
       <c r="D2" t="str">
         <v>1,548,000</v>
@@ -451,7 +451,7 @@
         <v>聖暉*</v>
       </c>
       <c r="C3" t="str">
-        <v>8.39%</v>
+        <v>8.06%</v>
       </c>
       <c r="D3" t="str">
         <v>3,355,000</v>
@@ -459,44 +459,44 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3105</v>
+        <v>6669</v>
       </c>
       <c r="B4" t="str">
-        <v>穩懋</v>
+        <v>緯穎</v>
       </c>
       <c r="C4" t="str">
-        <v>5.56%</v>
+        <v>6.21%</v>
       </c>
       <c r="D4" t="str">
-        <v>3,946,000</v>
+        <v>491,000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>6669</v>
+        <v>2383</v>
       </c>
       <c r="B5" t="str">
-        <v>緯穎</v>
+        <v>台光電</v>
       </c>
       <c r="C5" t="str">
-        <v>5.5%</v>
+        <v>5.59%</v>
       </c>
       <c r="D5" t="str">
-        <v>461,000</v>
+        <v>457,000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2383</v>
+        <v>3105</v>
       </c>
       <c r="B6" t="str">
-        <v>台光電</v>
+        <v>穩懋</v>
       </c>
       <c r="C6" t="str">
-        <v>5.26%</v>
+        <v>5.03%</v>
       </c>
       <c r="D6" t="str">
-        <v>457,000</v>
+        <v>3,946,000</v>
       </c>
     </row>
     <row r="7">
@@ -507,7 +507,7 @@
         <v>欣銓</v>
       </c>
       <c r="C7" t="str">
-        <v>4.37%</v>
+        <v>4.06%</v>
       </c>
       <c r="D7" t="str">
         <v>8,078,000</v>
@@ -515,16 +515,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6139</v>
+        <v>2345</v>
       </c>
       <c r="B8" t="str">
-        <v>亞翔</v>
+        <v>智邦</v>
       </c>
       <c r="C8" t="str">
-        <v>4.14%</v>
+        <v>4.05%</v>
       </c>
       <c r="D8" t="str">
-        <v>2,278,000</v>
+        <v>719,000</v>
       </c>
     </row>
     <row r="9">
@@ -535,7 +535,7 @@
         <v>奇鋐</v>
       </c>
       <c r="C9" t="str">
-        <v>4.08%</v>
+        <v>3.95%</v>
       </c>
       <c r="D9" t="str">
         <v>538,000</v>
@@ -543,44 +543,44 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2345</v>
+        <v>6139</v>
       </c>
       <c r="B10" t="str">
-        <v>智邦</v>
+        <v>亞翔</v>
       </c>
       <c r="C10" t="str">
-        <v>3.96%</v>
+        <v>3.93%</v>
       </c>
       <c r="D10" t="str">
-        <v>719,000</v>
+        <v>2,278,000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2308</v>
+        <v>2454</v>
       </c>
       <c r="B11" t="str">
-        <v>台達電</v>
+        <v>聯發科</v>
       </c>
       <c r="C11" t="str">
-        <v>3.68%</v>
+        <v>3.61%</v>
       </c>
       <c r="D11" t="str">
-        <v>690,000</v>
+        <v>573,000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2454</v>
+        <v>2308</v>
       </c>
       <c r="B12" t="str">
-        <v>聯發科</v>
+        <v>台達電</v>
       </c>
       <c r="C12" t="str">
-        <v>3.59%</v>
+        <v>3.61%</v>
       </c>
       <c r="D12" t="str">
-        <v>573,000</v>
+        <v>690,000</v>
       </c>
     </row>
     <row r="13">
@@ -591,7 +591,7 @@
         <v>致茂</v>
       </c>
       <c r="C13" t="str">
-        <v>3.58%</v>
+        <v>3.61%</v>
       </c>
       <c r="D13" t="str">
         <v>724,000</v>
@@ -605,7 +605,7 @@
         <v>旺矽</v>
       </c>
       <c r="C14" t="str">
-        <v>3.3%</v>
+        <v>3.49%</v>
       </c>
       <c r="D14" t="str">
         <v>276,000</v>
@@ -619,7 +619,7 @@
         <v>矽格</v>
       </c>
       <c r="C15" t="str">
-        <v>3.02%</v>
+        <v>2.92%</v>
       </c>
       <c r="D15" t="str">
         <v>6,338,000</v>
@@ -627,44 +627,44 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>6147</v>
+        <v>4958</v>
       </c>
       <c r="B16" t="str">
-        <v>頎邦</v>
+        <v>臻鼎-KY</v>
       </c>
       <c r="C16" t="str">
-        <v>2.44%</v>
+        <v>2.46%</v>
       </c>
       <c r="D16" t="str">
-        <v>6,546,000</v>
+        <v>2,654,000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>4958</v>
+        <v>3491</v>
       </c>
       <c r="B17" t="str">
-        <v>臻鼎-KY</v>
+        <v>昇達科</v>
       </c>
       <c r="C17" t="str">
-        <v>2.37%</v>
+        <v>2.24%</v>
       </c>
       <c r="D17" t="str">
-        <v>2,654,000</v>
+        <v>539,000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>3491</v>
+        <v>6147</v>
       </c>
       <c r="B18" t="str">
-        <v>昇達科</v>
+        <v>頎邦</v>
       </c>
       <c r="C18" t="str">
-        <v>2.18%</v>
+        <v>2.22%</v>
       </c>
       <c r="D18" t="str">
-        <v>539,000</v>
+        <v>6,546,000</v>
       </c>
     </row>
     <row r="19">
@@ -675,7 +675,7 @@
         <v>光洋科</v>
       </c>
       <c r="C19" t="str">
-        <v>1.73%</v>
+        <v>1.78%</v>
       </c>
       <c r="D19" t="str">
         <v>4,611,000</v>
@@ -689,38 +689,38 @@
         <v>富世達</v>
       </c>
       <c r="C20" t="str">
-        <v>1.68%</v>
+        <v>1.67%</v>
       </c>
       <c r="D20" t="str">
-        <v>341,000</v>
+        <v>311,000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2467</v>
+        <v>6285</v>
       </c>
       <c r="B21" t="str">
-        <v>志聖</v>
+        <v>啟碁</v>
       </c>
       <c r="C21" t="str">
-        <v>1.66%</v>
+        <v>1.64%</v>
       </c>
       <c r="D21" t="str">
-        <v>1,199,000</v>
+        <v>3,000,000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>6285</v>
+        <v>2467</v>
       </c>
       <c r="B22" t="str">
-        <v>啟碁</v>
+        <v>志聖</v>
       </c>
       <c r="C22" t="str">
-        <v>1.61%</v>
+        <v>1.54%</v>
       </c>
       <c r="D22" t="str">
-        <v>3,000,000</v>
+        <v>1,199,000</v>
       </c>
     </row>
     <row r="23">
@@ -731,7 +731,7 @@
         <v>精測</v>
       </c>
       <c r="C23" t="str">
-        <v>1.13%</v>
+        <v>1.12%</v>
       </c>
       <c r="D23" t="str">
         <v>121,000</v>
@@ -739,16 +739,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>8996</v>
+        <v>6488</v>
       </c>
       <c r="B24" t="str">
-        <v>高力</v>
+        <v>環球晶</v>
       </c>
       <c r="C24" t="str">
-        <v>1.08%</v>
+        <v>1.1%</v>
       </c>
       <c r="D24" t="str">
-        <v>373,000</v>
+        <v>683,000</v>
       </c>
     </row>
     <row r="25">
@@ -759,7 +759,7 @@
         <v>川湖</v>
       </c>
       <c r="C25" t="str">
-        <v>1.04%</v>
+        <v>1.09%</v>
       </c>
       <c r="D25" t="str">
         <v>106,000</v>
@@ -767,16 +767,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>6488</v>
+        <v>8996</v>
       </c>
       <c r="B26" t="str">
-        <v>環球晶</v>
+        <v>高力</v>
       </c>
       <c r="C26" t="str">
-        <v>1.02%</v>
+        <v>1.03%</v>
       </c>
       <c r="D26" t="str">
-        <v>683,000</v>
+        <v>373,000</v>
       </c>
     </row>
     <row r="27">
@@ -787,7 +787,7 @@
         <v>聯電</v>
       </c>
       <c r="C27" t="str">
-        <v>0.97%</v>
+        <v>0.95%</v>
       </c>
       <c r="D27" t="str">
         <v>5,045,000</v>
@@ -801,7 +801,7 @@
         <v>漢唐</v>
       </c>
       <c r="C28" t="str">
-        <v>0.94%</v>
+        <v>0.92%</v>
       </c>
       <c r="D28" t="str">
         <v>368,000</v>
@@ -823,30 +823,30 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2347</v>
+        <v>5289</v>
       </c>
       <c r="B30" t="str">
-        <v>聯強</v>
+        <v>宜鼎</v>
       </c>
       <c r="C30" t="str">
-        <v>0.79%</v>
+        <v>0.84%</v>
       </c>
       <c r="D30" t="str">
-        <v>3,693,000</v>
+        <v>274,000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>3583</v>
+        <v>3533</v>
       </c>
       <c r="B31" t="str">
-        <v>辛耘</v>
+        <v>嘉澤</v>
       </c>
       <c r="C31" t="str">
         <v>0.78%</v>
       </c>
       <c r="D31" t="str">
-        <v>370,000</v>
+        <v>111,000</v>
       </c>
     </row>
     <row r="32">
@@ -857,7 +857,7 @@
         <v>順達</v>
       </c>
       <c r="C32" t="str">
-        <v>0.77%</v>
+        <v>0.78%</v>
       </c>
       <c r="D32" t="str">
         <v>780,000</v>
@@ -865,30 +865,30 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>5289</v>
+        <v>2347</v>
       </c>
       <c r="B33" t="str">
-        <v>宜鼎</v>
+        <v>聯強</v>
       </c>
       <c r="C33" t="str">
         <v>0.77%</v>
       </c>
       <c r="D33" t="str">
-        <v>274,000</v>
+        <v>3,693,000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>3533</v>
+        <v>3583</v>
       </c>
       <c r="B34" t="str">
-        <v>嘉澤</v>
+        <v>辛耘</v>
       </c>
       <c r="C34" t="str">
-        <v>0.72%</v>
+        <v>0.7%</v>
       </c>
       <c r="D34" t="str">
-        <v>111,000</v>
+        <v>370,000</v>
       </c>
     </row>
     <row r="35">
@@ -899,7 +899,7 @@
         <v>弘塑</v>
       </c>
       <c r="C35" t="str">
-        <v>0.72%</v>
+        <v>0.66%</v>
       </c>
       <c r="D35" t="str">
         <v>89,000</v>
@@ -907,30 +907,30 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>6274</v>
+        <v>2313</v>
       </c>
       <c r="B36" t="str">
-        <v>台燿</v>
+        <v>華通</v>
       </c>
       <c r="C36" t="str">
-        <v>0.6%</v>
+        <v>0.63%</v>
       </c>
       <c r="D36" t="str">
-        <v>223,000</v>
+        <v>1,033,000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2313</v>
+        <v>6274</v>
       </c>
       <c r="B37" t="str">
-        <v>華通</v>
+        <v>台燿</v>
       </c>
       <c r="C37" t="str">
         <v>0.57%</v>
       </c>
       <c r="D37" t="str">
-        <v>1,033,000</v>
+        <v>223,000</v>
       </c>
     </row>
     <row r="38">
@@ -941,7 +941,7 @@
         <v>金像電</v>
       </c>
       <c r="C38" t="str">
-        <v>0.55%</v>
+        <v>0.57%</v>
       </c>
       <c r="D38" t="str">
         <v>155,000</v>
@@ -955,7 +955,7 @@
         <v>立隆電</v>
       </c>
       <c r="C39" t="str">
-        <v>0.54%</v>
+        <v>0.53%</v>
       </c>
       <c r="D39" t="str">
         <v>1,210,000</v>
@@ -983,7 +983,7 @@
         <v>貿聯-KY</v>
       </c>
       <c r="C41" t="str">
-        <v>0.41%</v>
+        <v>0.4%</v>
       </c>
       <c r="D41" t="str">
         <v>58,136</v>
@@ -991,30 +991,30 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>6691</v>
+        <v>4938</v>
       </c>
       <c r="B42" t="str">
-        <v>洋基工程</v>
+        <v>和碩</v>
       </c>
       <c r="C42" t="str">
-        <v>0.28%</v>
+        <v>0.27%</v>
       </c>
       <c r="D42" t="str">
-        <v>159,000</v>
+        <v>1,236,000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>4938</v>
+        <v>6691</v>
       </c>
       <c r="B43" t="str">
-        <v>和碩</v>
+        <v>洋基工程</v>
       </c>
       <c r="C43" t="str">
-        <v>0.27%</v>
+        <v>0.26%</v>
       </c>
       <c r="D43" t="str">
-        <v>1,236,000</v>
+        <v>159,000</v>
       </c>
     </row>
     <row r="44">
@@ -1039,7 +1039,7 @@
         <v>南電</v>
       </c>
       <c r="C45" t="str">
-        <v>0.23%</v>
+        <v>0.24%</v>
       </c>
       <c r="D45" t="str">
         <v>103,000</v>
@@ -1053,7 +1053,7 @@
         <v>力旺</v>
       </c>
       <c r="C46" t="str">
-        <v>0.23%</v>
+        <v>0.24%</v>
       </c>
       <c r="D46" t="str">
         <v>23,000</v>
@@ -1265,7 +1265,7 @@
         <v>債券附買回-P12遠傳1A</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD 10,001,800.00</v>
+        <v>TWD 10,003,589.00</v>
       </c>
     </row>
     <row r="3">
@@ -1300,7 +1300,7 @@
         <v>應收付證券款</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD 208,193,854.00</v>
+        <v>TWD 220,457,443.00</v>
       </c>
     </row>
     <row r="3">
@@ -1308,7 +1308,7 @@
         <v>現金</v>
       </c>
       <c r="B3" t="str">
-        <v>TWD 575,068,302.00</v>
+        <v>TWD 576,759,061.00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>